<commit_message>
tracking update 02.07.2026 20:15
</commit_message>
<xml_diff>
--- a/files/UAE-012_ФПЗ_24.06.2026.xlsx
+++ b/files/UAE-012_ФПЗ_24.06.2026.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\zinov\OneDrive\Desktop\РАБОЧАЯ\001 ИМПОРТ\001 containers\2026\001 UAE\UAE#12_VADIM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/7bb2b71721ea5021/Desktop/РАБОЧАЯ/001 ИМПОРТ/001 containers/2026/001 UAE/UAE#12_VADIM/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F48D7E9-18CD-46DD-9F95-25D0C0038AD4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{8F48D7E9-18CD-46DD-9F95-25D0C0038AD4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{695DD1DE-3592-47BC-8E23-ED1A771BB8DE}"/>
   <bookViews>
-    <workbookView xWindow="2475" yWindow="2235" windowWidth="35295" windowHeight="18060" tabRatio="611" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="611" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ФПЗ_Э12" sheetId="1" r:id="rId1"/>
@@ -1871,19 +1871,19 @@
         <v>22898.399999999998</v>
       </c>
       <c r="K2" s="24">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="L2" s="29">
         <f>H2*K2*1.0425</f>
-        <v>461.30624999999998</v>
+        <v>492.06</v>
       </c>
       <c r="M2" s="29">
         <f>$M$6/$I$4*I2</f>
-        <v>10779300</v>
+        <v>11497920</v>
       </c>
       <c r="N2" s="29">
         <f>$N$6/$I$4*I2</f>
-        <v>3233790</v>
+        <v>3449376</v>
       </c>
       <c r="O2" s="29">
         <f>$O$6/$J$4*J2</f>
@@ -1895,18 +1895,18 @@
       </c>
       <c r="Q2" s="29">
         <f t="shared" ref="Q2" si="1">M2+N2+O2+P2</f>
-        <v>15827196.53409091</v>
+        <v>16761402.53409091</v>
       </c>
       <c r="R2" s="30">
         <f>SUM(Q2/E2)</f>
-        <v>649.72071158008657</v>
+        <v>688.07071158008659</v>
       </c>
       <c r="S2" s="31">
         <v>717.3</v>
       </c>
       <c r="T2" s="32">
         <f>(S2-R2)/R2</f>
-        <v>0.10401282768955311</v>
+        <v>4.2480064807280025E-2</v>
       </c>
       <c r="U2" s="33">
         <f>S2*E2</f>
@@ -1914,7 +1914,7 @@
       </c>
       <c r="V2" s="33">
         <f t="shared" ref="V2" si="2">R2*E2</f>
-        <v>15827196.534090908</v>
+        <v>16761402.53409091</v>
       </c>
       <c r="W2" s="21"/>
       <c r="X2" s="21"/>
@@ -2941,7 +2941,7 @@
       </c>
       <c r="V3" s="41">
         <f>SUM(V2:V2)</f>
-        <v>15827196.534090908</v>
+        <v>16761402.53409091</v>
       </c>
       <c r="W3" s="21"/>
       <c r="X3" s="21"/>
@@ -2973,11 +2973,11 @@
       <c r="L4" s="7"/>
       <c r="M4" s="46">
         <f>SUMIF(M2:M2,"&lt;&gt;#ДЕЛ/0!")</f>
-        <v>10779300</v>
+        <v>11497920</v>
       </c>
       <c r="N4" s="46">
         <f>SUMIF(N2:N2,"&lt;&gt;#ДЕЛ/0!")</f>
-        <v>3233790</v>
+        <v>3449376</v>
       </c>
       <c r="O4" s="46">
         <f>SUMIF(O2:O2,"&lt;&gt;#ДЕЛ/0!")</f>
@@ -2989,7 +2989,7 @@
       </c>
       <c r="Q4" s="46">
         <f>SUMIF(Q2:Q2,"&lt;&gt;#ДЕЛ/0!")</f>
-        <v>15827196.53409091</v>
+        <v>16761402.53409091</v>
       </c>
       <c r="R4" s="47"/>
       <c r="S4" s="21"/>
@@ -3022,7 +3022,7 @@
       </c>
       <c r="V5" s="51">
         <f>(U3-V3)/V3</f>
-        <v>0.10401282768955324</v>
+        <v>4.2480064807280046E-2</v>
       </c>
     </row>
     <row r="6" spans="1:1019" ht="15.75" x14ac:dyDescent="0.25">
@@ -3030,11 +3030,11 @@
       <c r="J6" s="6"/>
       <c r="M6" s="52">
         <f>I4*K2</f>
-        <v>10779300</v>
+        <v>11497920</v>
       </c>
       <c r="N6" s="53">
         <f>M6*0.3</f>
-        <v>3233790</v>
+        <v>3449376</v>
       </c>
       <c r="O6" s="54">
         <v>1850000</v>
@@ -3044,11 +3044,11 @@
       </c>
       <c r="Q6" s="52">
         <f>M6+N6+O6+P6</f>
-        <v>15887090</v>
+        <v>16821296</v>
       </c>
       <c r="U6" s="41">
         <f>U3-V3</f>
-        <v>1646231.4659090918</v>
+        <v>712025.46590908989</v>
       </c>
     </row>
     <row r="7" spans="1:1019" x14ac:dyDescent="0.2">

</xml_diff>